<commit_message>
Add lithium carbonate forecast data
</commit_message>
<xml_diff>
--- a/lithium_carbonate_prediction_outputs/lithium_variable_forecast_report.xlsx
+++ b/lithium_carbonate_prediction_outputs/lithium_variable_forecast_report.xlsx
@@ -6842,31 +6842,31 @@
         <v>46235</v>
       </c>
       <c r="B2" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>11.28404669</v>
+        <v>10.54723031</v>
       </c>
       <c r="E2" t="n">
-        <v>114.4</v>
+        <v>116.1933333333333</v>
       </c>
       <c r="F2" t="n">
-        <v>1.100000000000008</v>
+        <v>2.046666666666673</v>
       </c>
       <c r="G2" t="n">
-        <v>1.1</v>
+        <v>2.046666666666667</v>
       </c>
       <c r="H2" t="n">
-        <v>1.070038910505855</v>
+        <v>2.02167575935958</v>
       </c>
       <c r="I2" t="n">
-        <v>118.2</v>
+        <v>121.6666666666666</v>
       </c>
       <c r="J2" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
     </row>
     <row r="3">
@@ -6874,31 +6874,31 @@
         <v>46266</v>
       </c>
       <c r="B3" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>11.28404669</v>
+        <v>10.15246153428571</v>
       </c>
       <c r="E3" t="n">
-        <v>114.4</v>
+        <v>116.4533333333333</v>
       </c>
       <c r="F3" t="n">
-        <v>1.100000000000008</v>
+        <v>2.340952380952389</v>
       </c>
       <c r="G3" t="n">
-        <v>1.1</v>
+        <v>2.340952380952381</v>
       </c>
       <c r="H3" t="n">
-        <v>1.070038910505855</v>
+        <v>2.309066814035366</v>
       </c>
       <c r="I3" t="n">
-        <v>118.2</v>
+        <v>124.0380952380952</v>
       </c>
       <c r="J3" t="n">
-        <v>170978.982923559</v>
+        <v>179801.4534453031</v>
       </c>
     </row>
     <row r="4">
@@ -6906,31 +6906,31 @@
         <v>46296</v>
       </c>
       <c r="B4" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>11.28404669</v>
+        <v>9.757692758571427</v>
       </c>
       <c r="E4" t="n">
-        <v>114.4</v>
+        <v>116.7133333333333</v>
       </c>
       <c r="F4" t="n">
-        <v>1.100000000000008</v>
+        <v>2.635238095238105</v>
       </c>
       <c r="G4" t="n">
-        <v>1.1</v>
+        <v>2.635238095238096</v>
       </c>
       <c r="H4" t="n">
-        <v>1.070038910505855</v>
+        <v>2.596457868711153</v>
       </c>
       <c r="I4" t="n">
-        <v>118.2</v>
+        <v>126.4095238095238</v>
       </c>
       <c r="J4" t="n">
-        <v>170978.982923559</v>
+        <v>187361.520936797</v>
       </c>
     </row>
     <row r="5">
@@ -6938,31 +6938,31 @@
         <v>46327</v>
       </c>
       <c r="B5" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>11.28404669</v>
+        <v>9.36292398285714</v>
       </c>
       <c r="E5" t="n">
-        <v>114.4</v>
+        <v>116.9733333333333</v>
       </c>
       <c r="F5" t="n">
-        <v>1.100000000000008</v>
+        <v>2.929523809523821</v>
       </c>
       <c r="G5" t="n">
-        <v>1.1</v>
+        <v>2.92952380952381</v>
       </c>
       <c r="H5" t="n">
-        <v>1.070038910505855</v>
+        <v>2.883848923386939</v>
       </c>
       <c r="I5" t="n">
-        <v>118.2</v>
+        <v>128.7809523809523</v>
       </c>
       <c r="J5" t="n">
-        <v>170978.982923559</v>
+        <v>194921.588428291</v>
       </c>
     </row>
     <row r="6">
@@ -6970,31 +6970,31 @@
         <v>46357</v>
       </c>
       <c r="B6" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>11.28404669</v>
+        <v>8.968155207142853</v>
       </c>
       <c r="E6" t="n">
-        <v>114.4</v>
+        <v>117.2333333333333</v>
       </c>
       <c r="F6" t="n">
-        <v>1.100000000000008</v>
+        <v>3.223809523809536</v>
       </c>
       <c r="G6" t="n">
-        <v>1.1</v>
+        <v>3.223809523809525</v>
       </c>
       <c r="H6" t="n">
-        <v>1.070038910505855</v>
+        <v>3.171239978062726</v>
       </c>
       <c r="I6" t="n">
-        <v>118.2</v>
+        <v>131.1523809523809</v>
       </c>
       <c r="J6" t="n">
-        <v>170978.982923559</v>
+        <v>202481.6559197848</v>
       </c>
     </row>
   </sheetData>
@@ -17230,35 +17230,35 @@
         <v>46204</v>
       </c>
       <c r="C2" t="n">
-        <v>30.79693624030095</v>
+        <v>28.98535175557737</v>
       </c>
       <c r="D2" t="n">
-        <v>40.57880515023948</v>
+        <v>38.1918166119901</v>
       </c>
       <c r="E2" t="n">
-        <v>11.28404669</v>
+        <v>11.21748285731092</v>
       </c>
       <c r="F2" t="n">
-        <v>114.4</v>
+        <v>114.5207843137255</v>
       </c>
       <c r="G2" t="n">
-        <v>1.100000000000008</v>
+        <v>1.17299719887956</v>
       </c>
       <c r="H2" t="n">
-        <v>1.1</v>
+        <v>1.172997198879552</v>
       </c>
       <c r="I2" t="n">
-        <v>1.070038910505855</v>
+        <v>1.14292290483112</v>
       </c>
       <c r="J2" t="n">
-        <v>118.2</v>
+        <v>118.5434173669468</v>
       </c>
       <c r="K2" t="n">
-        <v>172741.5735410651</v>
+        <v>173403.7819613006</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>172741.5735410651</v>
+        <v>173403.7819613006</v>
       </c>
     </row>
     <row r="3">
@@ -17269,35 +17269,35 @@
         <v>46204</v>
       </c>
       <c r="C3" t="n">
-        <v>30.79693624030095</v>
+        <v>27.17376727085378</v>
       </c>
       <c r="D3" t="n">
-        <v>40.57880515023948</v>
+        <v>35.80482807374072</v>
       </c>
       <c r="E3" t="n">
-        <v>11.28404669</v>
+        <v>11.15091902462185</v>
       </c>
       <c r="F3" t="n">
-        <v>114.4</v>
+        <v>114.641568627451</v>
       </c>
       <c r="G3" t="n">
-        <v>1.100000000000008</v>
+        <v>1.245994397759112</v>
       </c>
       <c r="H3" t="n">
-        <v>1.1</v>
+        <v>1.245994397759104</v>
       </c>
       <c r="I3" t="n">
-        <v>1.070038910505855</v>
+        <v>1.215806899156386</v>
       </c>
       <c r="J3" t="n">
-        <v>118.2</v>
+        <v>118.8868347338936</v>
       </c>
       <c r="K3" t="n">
-        <v>172741.5735410651</v>
+        <v>174065.9903815364</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>172741.5735410651</v>
+        <v>174065.9903815364</v>
       </c>
     </row>
     <row r="4">
@@ -17308,35 +17308,35 @@
         <v>46204</v>
       </c>
       <c r="C4" t="n">
-        <v>30.79693624030095</v>
+        <v>21.73901381668303</v>
       </c>
       <c r="D4" t="n">
-        <v>40.57880515023948</v>
+        <v>28.64386245899258</v>
       </c>
       <c r="E4" t="n">
-        <v>11.28404669</v>
+        <v>10.95122752655462</v>
       </c>
       <c r="F4" t="n">
-        <v>114.4</v>
+        <v>115.0039215686274</v>
       </c>
       <c r="G4" t="n">
-        <v>1.100000000000008</v>
+        <v>1.464985994397767</v>
       </c>
       <c r="H4" t="n">
-        <v>1.1</v>
+        <v>1.464985994397759</v>
       </c>
       <c r="I4" t="n">
-        <v>1.070038910505855</v>
+        <v>1.434458882132182</v>
       </c>
       <c r="J4" t="n">
-        <v>118.2</v>
+        <v>119.9170868347339</v>
       </c>
       <c r="K4" t="n">
-        <v>172741.5735410651</v>
+        <v>176052.6156422432</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>172741.5735410651</v>
+        <v>176052.6156422432</v>
       </c>
     </row>
     <row r="5">
@@ -17347,35 +17347,35 @@
         <v>46204</v>
       </c>
       <c r="C5" t="n">
-        <v>30.79693624030095</v>
+        <v>19.92742933195944</v>
       </c>
       <c r="D5" t="n">
-        <v>40.57880515023948</v>
+        <v>26.2568739207432</v>
       </c>
       <c r="E5" t="n">
-        <v>11.28404669</v>
+        <v>10.88466369386555</v>
       </c>
       <c r="F5" t="n">
-        <v>114.4</v>
+        <v>115.1247058823529</v>
       </c>
       <c r="G5" t="n">
-        <v>1.100000000000008</v>
+        <v>1.537983193277319</v>
       </c>
       <c r="H5" t="n">
-        <v>1.1</v>
+        <v>1.537983193277311</v>
       </c>
       <c r="I5" t="n">
-        <v>1.070038910505855</v>
+        <v>1.507342876457447</v>
       </c>
       <c r="J5" t="n">
-        <v>118.2</v>
+        <v>120.2605042016807</v>
       </c>
       <c r="K5" t="n">
-        <v>172741.5735410651</v>
+        <v>176714.8240624789</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
-        <v>172741.5735410651</v>
+        <v>176714.8240624789</v>
       </c>
     </row>
     <row r="6">
@@ -17386,35 +17386,35 @@
         <v>46204</v>
       </c>
       <c r="C6" t="n">
-        <v>30.79693624030095</v>
+        <v>18.11584484723586</v>
       </c>
       <c r="D6" t="n">
-        <v>40.57880515023948</v>
+        <v>23.86988538249381</v>
       </c>
       <c r="E6" t="n">
-        <v>11.28404669</v>
+        <v>10.81809986117647</v>
       </c>
       <c r="F6" t="n">
-        <v>114.4</v>
+        <v>115.2454901960784</v>
       </c>
       <c r="G6" t="n">
-        <v>1.100000000000008</v>
+        <v>1.610980392156871</v>
       </c>
       <c r="H6" t="n">
-        <v>1.1</v>
+        <v>1.610980392156863</v>
       </c>
       <c r="I6" t="n">
-        <v>1.070038910505855</v>
+        <v>1.580226870782713</v>
       </c>
       <c r="J6" t="n">
-        <v>118.2</v>
+        <v>120.6039215686274</v>
       </c>
       <c r="K6" t="n">
-        <v>172741.5735410651</v>
+        <v>177377.0324827145</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>172741.5735410651</v>
+        <v>177377.0324827145</v>
       </c>
     </row>
     <row r="7">
@@ -17425,35 +17425,35 @@
         <v>46204</v>
       </c>
       <c r="C7" t="n">
-        <v>30.79693624030095</v>
+        <v>16.30426036251227</v>
       </c>
       <c r="D7" t="n">
-        <v>40.57880515023948</v>
+        <v>21.48289684424443</v>
       </c>
       <c r="E7" t="n">
-        <v>11.28404669</v>
+        <v>10.7515360284874</v>
       </c>
       <c r="F7" t="n">
-        <v>114.4</v>
+        <v>115.3662745098039</v>
       </c>
       <c r="G7" t="n">
-        <v>1.100000000000008</v>
+        <v>1.683977591036423</v>
       </c>
       <c r="H7" t="n">
-        <v>1.1</v>
+        <v>1.683977591036415</v>
       </c>
       <c r="I7" t="n">
-        <v>1.070038910505855</v>
+        <v>1.653110865107978</v>
       </c>
       <c r="J7" t="n">
-        <v>118.2</v>
+        <v>120.9473389355742</v>
       </c>
       <c r="K7" t="n">
-        <v>172741.5735410651</v>
+        <v>178039.2409029503</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>172741.5735410651</v>
+        <v>178039.2409029503</v>
       </c>
     </row>
     <row r="8">
@@ -17464,35 +17464,35 @@
         <v>46204</v>
       </c>
       <c r="C8" t="n">
-        <v>30.79693624030095</v>
+        <v>14.49267587778868</v>
       </c>
       <c r="D8" t="n">
-        <v>40.57880515023948</v>
+        <v>19.09590830599505</v>
       </c>
       <c r="E8" t="n">
-        <v>11.28404669</v>
+        <v>10.68497219579832</v>
       </c>
       <c r="F8" t="n">
-        <v>114.4</v>
+        <v>115.4870588235294</v>
       </c>
       <c r="G8" t="n">
-        <v>1.100000000000008</v>
+        <v>1.756974789915974</v>
       </c>
       <c r="H8" t="n">
-        <v>1.1</v>
+        <v>1.756974789915966</v>
       </c>
       <c r="I8" t="n">
-        <v>1.070038910505855</v>
+        <v>1.725994859433243</v>
       </c>
       <c r="J8" t="n">
-        <v>118.2</v>
+        <v>121.290756302521</v>
       </c>
       <c r="K8" t="n">
-        <v>172741.5735410651</v>
+        <v>178701.4493231857</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
-        <v>172741.5735410651</v>
+        <v>178701.4493231857</v>
       </c>
     </row>
     <row r="9">
@@ -17503,35 +17503,35 @@
         <v>46204</v>
       </c>
       <c r="C9" t="n">
-        <v>30.79693624030095</v>
+        <v>9.057922423617928</v>
       </c>
       <c r="D9" t="n">
-        <v>40.57880515023948</v>
+        <v>11.93494269124691</v>
       </c>
       <c r="E9" t="n">
-        <v>11.28404669</v>
+        <v>10.48528069773109</v>
       </c>
       <c r="F9" t="n">
-        <v>114.4</v>
+        <v>115.8494117647058</v>
       </c>
       <c r="G9" t="n">
-        <v>1.100000000000008</v>
+        <v>1.97596638655463</v>
       </c>
       <c r="H9" t="n">
-        <v>1.1</v>
+        <v>1.975966386554622</v>
       </c>
       <c r="I9" t="n">
-        <v>1.070038910505855</v>
+        <v>1.94464684240904</v>
       </c>
       <c r="J9" t="n">
-        <v>118.2</v>
+        <v>122.3210084033613</v>
       </c>
       <c r="K9" t="n">
-        <v>172741.5735410651</v>
+        <v>180688.0745838928</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>172741.5735410651</v>
+        <v>180688.0745838928</v>
       </c>
     </row>
     <row r="10">
@@ -17542,35 +17542,35 @@
         <v>46204</v>
       </c>
       <c r="C10" t="n">
-        <v>30.79693624030095</v>
+        <v>7.246337938894342</v>
       </c>
       <c r="D10" t="n">
-        <v>40.57880515023948</v>
+        <v>9.547954152997526</v>
       </c>
       <c r="E10" t="n">
-        <v>11.28404669</v>
+        <v>10.41871686504202</v>
       </c>
       <c r="F10" t="n">
-        <v>114.4</v>
+        <v>115.9701960784313</v>
       </c>
       <c r="G10" t="n">
-        <v>1.100000000000008</v>
+        <v>2.048963585434182</v>
       </c>
       <c r="H10" t="n">
-        <v>1.1</v>
+        <v>2.048963585434174</v>
       </c>
       <c r="I10" t="n">
-        <v>1.070038910505855</v>
+        <v>2.017530836734305</v>
       </c>
       <c r="J10" t="n">
-        <v>118.2</v>
+        <v>122.6644257703081</v>
       </c>
       <c r="K10" t="n">
-        <v>172741.5735410651</v>
+        <v>181350.2830041284</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>172741.5735410651</v>
+        <v>181350.2830041284</v>
       </c>
     </row>
     <row r="11">
@@ -17581,35 +17581,35 @@
         <v>46204</v>
       </c>
       <c r="C11" t="n">
-        <v>30.79693624030095</v>
+        <v>5.434753454170757</v>
       </c>
       <c r="D11" t="n">
-        <v>40.57880515023948</v>
+        <v>7.160965614748143</v>
       </c>
       <c r="E11" t="n">
-        <v>11.28404669</v>
+        <v>10.35215303235294</v>
       </c>
       <c r="F11" t="n">
-        <v>114.4</v>
+        <v>116.0909803921568</v>
       </c>
       <c r="G11" t="n">
-        <v>1.100000000000008</v>
+        <v>2.121960784313734</v>
       </c>
       <c r="H11" t="n">
-        <v>1.1</v>
+        <v>2.121960784313726</v>
       </c>
       <c r="I11" t="n">
-        <v>1.070038910505855</v>
+        <v>2.09041483105957</v>
       </c>
       <c r="J11" t="n">
-        <v>118.2</v>
+        <v>123.0078431372549</v>
       </c>
       <c r="K11" t="n">
-        <v>172741.5735410651</v>
+        <v>182012.4914243641</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>172741.5735410651</v>
+        <v>182012.4914243641</v>
       </c>
     </row>
     <row r="12">
@@ -17620,35 +17620,35 @@
         <v>46204</v>
       </c>
       <c r="C12" t="n">
-        <v>30.79693624030095</v>
+        <v>3.623168969447171</v>
       </c>
       <c r="D12" t="n">
-        <v>40.57880515023948</v>
+        <v>4.773977076498767</v>
       </c>
       <c r="E12" t="n">
-        <v>11.28404669</v>
+        <v>10.28558919966386</v>
       </c>
       <c r="F12" t="n">
-        <v>114.4</v>
+        <v>116.2117647058823</v>
       </c>
       <c r="G12" t="n">
-        <v>1.100000000000008</v>
+        <v>2.194957983193286</v>
       </c>
       <c r="H12" t="n">
-        <v>1.1</v>
+        <v>2.194957983193278</v>
       </c>
       <c r="I12" t="n">
-        <v>1.070038910505855</v>
+        <v>2.163298825384835</v>
       </c>
       <c r="J12" t="n">
-        <v>118.2</v>
+        <v>123.3512605042016</v>
       </c>
       <c r="K12" t="n">
-        <v>172741.5735410651</v>
+        <v>182674.6998445996</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>172741.5735410651</v>
+        <v>182674.6998445996</v>
       </c>
     </row>
     <row r="13">
@@ -17659,35 +17659,35 @@
         <v>46204</v>
       </c>
       <c r="C13" t="n">
-        <v>30.79693624030095</v>
+        <v>1.811584484723586</v>
       </c>
       <c r="D13" t="n">
-        <v>40.57880515023948</v>
+        <v>2.386988538249383</v>
       </c>
       <c r="E13" t="n">
-        <v>11.28404669</v>
+        <v>10.21902536697479</v>
       </c>
       <c r="F13" t="n">
-        <v>114.4</v>
+        <v>116.3325490196078</v>
       </c>
       <c r="G13" t="n">
-        <v>1.100000000000008</v>
+        <v>2.267955182072837</v>
       </c>
       <c r="H13" t="n">
-        <v>1.1</v>
+        <v>2.267955182072829</v>
       </c>
       <c r="I13" t="n">
-        <v>1.070038910505855</v>
+        <v>2.236182819710101</v>
       </c>
       <c r="J13" t="n">
-        <v>118.2</v>
+        <v>123.6946778711484</v>
       </c>
       <c r="K13" t="n">
-        <v>172741.5735410651</v>
+        <v>183336.9082648353</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>172741.5735410651</v>
+        <v>183336.9082648353</v>
       </c>
     </row>
     <row r="14">
@@ -17698,37 +17698,37 @@
         <v>46235</v>
       </c>
       <c r="C14" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>11.28404669</v>
+        <v>10.12699258101382</v>
       </c>
       <c r="F14" t="n">
-        <v>114.4</v>
+        <v>116.4701075268817</v>
       </c>
       <c r="G14" t="n">
-        <v>1.100000000000008</v>
+        <v>2.359938556067597</v>
       </c>
       <c r="H14" t="n">
-        <v>1.1</v>
+        <v>2.359938556067589</v>
       </c>
       <c r="I14" t="n">
-        <v>1.070038910505855</v>
+        <v>2.327608172401546</v>
       </c>
       <c r="J14" t="n">
-        <v>118.2</v>
+        <v>124.1910906298003</v>
       </c>
       <c r="K14" t="n">
-        <v>172741.5735410651</v>
+        <v>184533.0605795599</v>
       </c>
       <c r="L14" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M14" t="n">
-        <v>170978.9829235589</v>
+        <v>169260.1992095786</v>
       </c>
     </row>
     <row r="15">
@@ -17739,37 +17739,37 @@
         <v>46235</v>
       </c>
       <c r="C15" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>11.28404669</v>
+        <v>10.11425810437788</v>
       </c>
       <c r="F15" t="n">
-        <v>114.4</v>
+        <v>116.4784946236559</v>
       </c>
       <c r="G15" t="n">
-        <v>1.100000000000008</v>
+        <v>2.3694316436252</v>
       </c>
       <c r="H15" t="n">
-        <v>1.1</v>
+        <v>2.369431643625192</v>
       </c>
       <c r="I15" t="n">
-        <v>1.070038910505855</v>
+        <v>2.336878851584636</v>
       </c>
       <c r="J15" t="n">
-        <v>118.2</v>
+        <v>124.2675883256528</v>
       </c>
       <c r="K15" t="n">
-        <v>172741.5735410651</v>
+        <v>184800.0325268043</v>
       </c>
       <c r="L15" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M15" t="n">
-        <v>170978.9829235589</v>
+        <v>169527.171156823</v>
       </c>
     </row>
     <row r="16">
@@ -17780,37 +17780,37 @@
         <v>46235</v>
       </c>
       <c r="C16" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>11.28404669</v>
+        <v>10.10152362774194</v>
       </c>
       <c r="F16" t="n">
-        <v>114.4</v>
+        <v>116.4868817204301</v>
       </c>
       <c r="G16" t="n">
-        <v>1.100000000000008</v>
+        <v>2.378924731182804</v>
       </c>
       <c r="H16" t="n">
-        <v>1.1</v>
+        <v>2.378924731182796</v>
       </c>
       <c r="I16" t="n">
-        <v>1.070038910505855</v>
+        <v>2.346149530767726</v>
       </c>
       <c r="J16" t="n">
-        <v>118.2</v>
+        <v>124.3440860215053</v>
       </c>
       <c r="K16" t="n">
-        <v>172741.5735410651</v>
+        <v>185067.004474049</v>
       </c>
       <c r="L16" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M16" t="n">
-        <v>170978.9829235589</v>
+        <v>169794.1431040677</v>
       </c>
     </row>
     <row r="17">
@@ -17821,37 +17821,37 @@
         <v>46235</v>
       </c>
       <c r="C17" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>11.28404669</v>
+        <v>10.08878915110599</v>
       </c>
       <c r="F17" t="n">
-        <v>114.4</v>
+        <v>116.4952688172043</v>
       </c>
       <c r="G17" t="n">
-        <v>1.100000000000008</v>
+        <v>2.388417818740407</v>
       </c>
       <c r="H17" t="n">
-        <v>1.1</v>
+        <v>2.3884178187404</v>
       </c>
       <c r="I17" t="n">
-        <v>1.070038910505855</v>
+        <v>2.355420209950816</v>
       </c>
       <c r="J17" t="n">
-        <v>118.2</v>
+        <v>124.4205837173579</v>
       </c>
       <c r="K17" t="n">
-        <v>172741.5735410651</v>
+        <v>185333.9764212934</v>
       </c>
       <c r="L17" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M17" t="n">
-        <v>170978.9829235589</v>
+        <v>170061.1150513121</v>
       </c>
     </row>
     <row r="18">
@@ -17862,37 +17862,37 @@
         <v>46235</v>
       </c>
       <c r="C18" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>11.28404669</v>
+        <v>10.07605467447005</v>
       </c>
       <c r="F18" t="n">
-        <v>114.4</v>
+        <v>116.5036559139784</v>
       </c>
       <c r="G18" t="n">
-        <v>1.100000000000008</v>
+        <v>2.397910906298011</v>
       </c>
       <c r="H18" t="n">
-        <v>1.1</v>
+        <v>2.397910906298003</v>
       </c>
       <c r="I18" t="n">
-        <v>1.070038910505855</v>
+        <v>2.364690889133906</v>
       </c>
       <c r="J18" t="n">
-        <v>118.2</v>
+        <v>124.4970814132104</v>
       </c>
       <c r="K18" t="n">
-        <v>172741.5735410651</v>
+        <v>185600.948368538</v>
       </c>
       <c r="L18" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M18" t="n">
-        <v>170978.9829235589</v>
+        <v>170328.0869985567</v>
       </c>
     </row>
     <row r="19">
@@ -17903,37 +17903,37 @@
         <v>46235</v>
       </c>
       <c r="C19" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>11.28404669</v>
+        <v>10.03785124456221</v>
       </c>
       <c r="F19" t="n">
-        <v>114.4</v>
+        <v>116.528817204301</v>
       </c>
       <c r="G19" t="n">
-        <v>1.100000000000008</v>
+        <v>2.426390168970823</v>
       </c>
       <c r="H19" t="n">
-        <v>1.1</v>
+        <v>2.426390168970815</v>
       </c>
       <c r="I19" t="n">
-        <v>1.070038910505855</v>
+        <v>2.392502926683175</v>
       </c>
       <c r="J19" t="n">
-        <v>118.2</v>
+        <v>124.726574500768</v>
       </c>
       <c r="K19" t="n">
-        <v>172741.5735410651</v>
+        <v>186401.8642102715</v>
       </c>
       <c r="L19" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M19" t="n">
-        <v>170978.9829235589</v>
+        <v>171129.0028402902</v>
       </c>
     </row>
     <row r="20">
@@ -17944,37 +17944,37 @@
         <v>46235</v>
       </c>
       <c r="C20" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>11.28404669</v>
+        <v>10.02511676792627</v>
       </c>
       <c r="F20" t="n">
-        <v>114.4</v>
+        <v>116.5372043010752</v>
       </c>
       <c r="G20" t="n">
-        <v>1.100000000000008</v>
+        <v>2.435883256528426</v>
       </c>
       <c r="H20" t="n">
-        <v>1.1</v>
+        <v>2.435883256528418</v>
       </c>
       <c r="I20" t="n">
-        <v>1.070038910505855</v>
+        <v>2.401773605866265</v>
       </c>
       <c r="J20" t="n">
-        <v>118.2</v>
+        <v>124.8030721966205</v>
       </c>
       <c r="K20" t="n">
-        <v>172741.5735410651</v>
+        <v>186668.836157516</v>
       </c>
       <c r="L20" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M20" t="n">
-        <v>170978.9829235589</v>
+        <v>171395.9747875347</v>
       </c>
     </row>
     <row r="21">
@@ -17985,37 +17985,37 @@
         <v>46235</v>
       </c>
       <c r="C21" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>11.28404669</v>
+        <v>10.01238229129032</v>
       </c>
       <c r="F21" t="n">
-        <v>114.4</v>
+        <v>116.5455913978494</v>
       </c>
       <c r="G21" t="n">
-        <v>1.100000000000008</v>
+        <v>2.44537634408603</v>
       </c>
       <c r="H21" t="n">
-        <v>1.1</v>
+        <v>2.445376344086022</v>
       </c>
       <c r="I21" t="n">
-        <v>1.070038910505855</v>
+        <v>2.411044285049355</v>
       </c>
       <c r="J21" t="n">
-        <v>118.2</v>
+        <v>124.8795698924731</v>
       </c>
       <c r="K21" t="n">
-        <v>172741.5735410651</v>
+        <v>186935.8081047605</v>
       </c>
       <c r="L21" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M21" t="n">
-        <v>170978.9829235589</v>
+        <v>171662.9467347792</v>
       </c>
     </row>
     <row r="22">
@@ -18026,37 +18026,37 @@
         <v>46235</v>
       </c>
       <c r="C22" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>11.28404669</v>
+        <v>9.999647814654377</v>
       </c>
       <c r="F22" t="n">
-        <v>114.4</v>
+        <v>116.5539784946236</v>
       </c>
       <c r="G22" t="n">
-        <v>1.100000000000008</v>
+        <v>2.454869431643634</v>
       </c>
       <c r="H22" t="n">
-        <v>1.1</v>
+        <v>2.454869431643626</v>
       </c>
       <c r="I22" t="n">
-        <v>1.070038910505855</v>
+        <v>2.420314964232445</v>
       </c>
       <c r="J22" t="n">
-        <v>118.2</v>
+        <v>124.9560675883256</v>
       </c>
       <c r="K22" t="n">
-        <v>172741.5735410651</v>
+        <v>187202.7800520051</v>
       </c>
       <c r="L22" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M22" t="n">
-        <v>170978.9829235589</v>
+        <v>171929.9186820238</v>
       </c>
     </row>
     <row r="23">
@@ -18067,37 +18067,37 @@
         <v>46235</v>
       </c>
       <c r="C23" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>11.28404669</v>
+        <v>9.986913338018432</v>
       </c>
       <c r="F23" t="n">
-        <v>114.4</v>
+        <v>116.5623655913978</v>
       </c>
       <c r="G23" t="n">
-        <v>1.100000000000008</v>
+        <v>2.464362519201238</v>
       </c>
       <c r="H23" t="n">
-        <v>1.1</v>
+        <v>2.46436251920123</v>
       </c>
       <c r="I23" t="n">
-        <v>1.070038910505855</v>
+        <v>2.429585643415535</v>
       </c>
       <c r="J23" t="n">
-        <v>118.2</v>
+        <v>125.0325652841781</v>
       </c>
       <c r="K23" t="n">
-        <v>172741.5735410651</v>
+        <v>187469.7519992497</v>
       </c>
       <c r="L23" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M23" t="n">
-        <v>170978.9829235589</v>
+        <v>172196.8906292683</v>
       </c>
     </row>
     <row r="24">
@@ -18108,37 +18108,37 @@
         <v>46235</v>
       </c>
       <c r="C24" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>11.28404669</v>
+        <v>9.948709908110597</v>
       </c>
       <c r="F24" t="n">
-        <v>114.4</v>
+        <v>116.5875268817204</v>
       </c>
       <c r="G24" t="n">
-        <v>1.100000000000008</v>
+        <v>2.492841781874048</v>
       </c>
       <c r="H24" t="n">
-        <v>1.1</v>
+        <v>2.49284178187404</v>
       </c>
       <c r="I24" t="n">
-        <v>1.070038910505855</v>
+        <v>2.457397680964804</v>
       </c>
       <c r="J24" t="n">
-        <v>118.2</v>
+        <v>125.2620583717357</v>
       </c>
       <c r="K24" t="n">
-        <v>172741.5735410651</v>
+        <v>188270.6678409832</v>
       </c>
       <c r="L24" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M24" t="n">
-        <v>170978.9829235589</v>
+        <v>172997.8064710019</v>
       </c>
     </row>
     <row r="25">
@@ -18149,37 +18149,37 @@
         <v>46235</v>
       </c>
       <c r="C25" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>11.28404669</v>
+        <v>9.935975431474652</v>
       </c>
       <c r="F25" t="n">
-        <v>114.4</v>
+        <v>116.5959139784946</v>
       </c>
       <c r="G25" t="n">
-        <v>1.100000000000008</v>
+        <v>2.502334869431652</v>
       </c>
       <c r="H25" t="n">
-        <v>1.1</v>
+        <v>2.502334869431644</v>
       </c>
       <c r="I25" t="n">
-        <v>1.070038910505855</v>
+        <v>2.466668360147894</v>
       </c>
       <c r="J25" t="n">
-        <v>118.2</v>
+        <v>125.3385560675883</v>
       </c>
       <c r="K25" t="n">
-        <v>172741.5735410651</v>
+        <v>188537.6397882277</v>
       </c>
       <c r="L25" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M25" t="n">
-        <v>170978.9829235589</v>
+        <v>173264.7784182463</v>
       </c>
     </row>
     <row r="26">
@@ -18190,37 +18190,37 @@
         <v>46235</v>
       </c>
       <c r="C26" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>11.28404669</v>
+        <v>9.923240954838707</v>
       </c>
       <c r="F26" t="n">
-        <v>114.4</v>
+        <v>116.6043010752688</v>
       </c>
       <c r="G26" t="n">
-        <v>1.100000000000008</v>
+        <v>2.511827956989256</v>
       </c>
       <c r="H26" t="n">
-        <v>1.1</v>
+        <v>2.511827956989248</v>
       </c>
       <c r="I26" t="n">
-        <v>1.070038910505855</v>
+        <v>2.475939039330984</v>
       </c>
       <c r="J26" t="n">
-        <v>118.2</v>
+        <v>125.4150537634408</v>
       </c>
       <c r="K26" t="n">
-        <v>172741.5735410651</v>
+        <v>188804.6117354723</v>
       </c>
       <c r="L26" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M26" t="n">
-        <v>170978.9829235589</v>
+        <v>173531.7503654909</v>
       </c>
     </row>
     <row r="27">
@@ -18231,37 +18231,37 @@
         <v>46235</v>
       </c>
       <c r="C27" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>11.28404669</v>
+        <v>9.910506478202763</v>
       </c>
       <c r="F27" t="n">
-        <v>114.4</v>
+        <v>116.612688172043</v>
       </c>
       <c r="G27" t="n">
-        <v>1.100000000000008</v>
+        <v>2.52132104454686</v>
       </c>
       <c r="H27" t="n">
-        <v>1.1</v>
+        <v>2.521321044546851</v>
       </c>
       <c r="I27" t="n">
-        <v>1.070038910505855</v>
+        <v>2.485209718514074</v>
       </c>
       <c r="J27" t="n">
-        <v>118.2</v>
+        <v>125.4915514592933</v>
       </c>
       <c r="K27" t="n">
-        <v>172741.5735410651</v>
+        <v>189071.5836827167</v>
       </c>
       <c r="L27" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M27" t="n">
-        <v>170978.9829235589</v>
+        <v>173798.7223127354</v>
       </c>
     </row>
     <row r="28">
@@ -18272,37 +18272,37 @@
         <v>46235</v>
       </c>
       <c r="C28" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>11.28404669</v>
+        <v>9.897772001566819</v>
       </c>
       <c r="F28" t="n">
-        <v>114.4</v>
+        <v>116.6210752688172</v>
       </c>
       <c r="G28" t="n">
-        <v>1.100000000000008</v>
+        <v>2.530814132104464</v>
       </c>
       <c r="H28" t="n">
-        <v>1.1</v>
+        <v>2.530814132104455</v>
       </c>
       <c r="I28" t="n">
-        <v>1.070038910505855</v>
+        <v>2.494480397697164</v>
       </c>
       <c r="J28" t="n">
-        <v>118.2</v>
+        <v>125.5680491551459</v>
       </c>
       <c r="K28" t="n">
-        <v>172741.5735410651</v>
+        <v>189338.5556299614</v>
       </c>
       <c r="L28" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M28" t="n">
-        <v>170978.9829235589</v>
+        <v>174065.6942599801</v>
       </c>
     </row>
     <row r="29">
@@ -18313,37 +18313,37 @@
         <v>46235</v>
       </c>
       <c r="C29" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>11.28404669</v>
+        <v>9.859568571658984</v>
       </c>
       <c r="F29" t="n">
-        <v>114.4</v>
+        <v>116.6462365591397</v>
       </c>
       <c r="G29" t="n">
-        <v>1.100000000000008</v>
+        <v>2.559293394777275</v>
       </c>
       <c r="H29" t="n">
-        <v>1.1</v>
+        <v>2.559293394777266</v>
       </c>
       <c r="I29" t="n">
-        <v>1.070038910505855</v>
+        <v>2.522292435246434</v>
       </c>
       <c r="J29" t="n">
-        <v>118.2</v>
+        <v>125.7975422427035</v>
       </c>
       <c r="K29" t="n">
-        <v>172741.5735410651</v>
+        <v>190139.4714716948</v>
       </c>
       <c r="L29" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M29" t="n">
-        <v>170978.9829235589</v>
+        <v>174866.6101017135</v>
       </c>
     </row>
     <row r="30">
@@ -18354,37 +18354,37 @@
         <v>46235</v>
       </c>
       <c r="C30" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>11.28404669</v>
+        <v>9.84683409502304</v>
       </c>
       <c r="F30" t="n">
-        <v>114.4</v>
+        <v>116.6546236559139</v>
       </c>
       <c r="G30" t="n">
-        <v>1.100000000000008</v>
+        <v>2.568786482334878</v>
       </c>
       <c r="H30" t="n">
-        <v>1.1</v>
+        <v>2.56878648233487</v>
       </c>
       <c r="I30" t="n">
-        <v>1.070038910505855</v>
+        <v>2.531563114429523</v>
       </c>
       <c r="J30" t="n">
-        <v>118.2</v>
+        <v>125.874039938556</v>
       </c>
       <c r="K30" t="n">
-        <v>172741.5735410651</v>
+        <v>190406.4434189393</v>
       </c>
       <c r="L30" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M30" t="n">
-        <v>170978.9829235589</v>
+        <v>175133.582048958</v>
       </c>
     </row>
     <row r="31">
@@ -18395,37 +18395,37 @@
         <v>46235</v>
       </c>
       <c r="C31" t="n">
-        <v>30.79693624030095</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>40.57880515023948</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>11.28404669</v>
+        <v>9.834099618387095</v>
       </c>
       <c r="F31" t="n">
-        <v>114.4</v>
+        <v>116.6630107526881</v>
       </c>
       <c r="G31" t="n">
-        <v>1.100000000000008</v>
+        <v>2.578279569892482</v>
       </c>
       <c r="H31" t="n">
-        <v>1.1</v>
+        <v>2.578279569892474</v>
       </c>
       <c r="I31" t="n">
-        <v>1.070038910505855</v>
+        <v>2.540833793612614</v>
       </c>
       <c r="J31" t="n">
-        <v>118.2</v>
+        <v>125.9505376344086</v>
       </c>
       <c r="K31" t="n">
-        <v>172741.5735410651</v>
+        <v>190673.4153661839</v>
       </c>
       <c r="L31" t="n">
-        <v>170978.982923559</v>
+        <v>172241.385953809</v>
       </c>
       <c r="M31" t="n">
-        <v>170978.9829235589</v>
+        <v>175400.5539962026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>